<commit_message>
Fix tablero proyeccion (auth_check) + actualizar tableros
</commit_message>
<xml_diff>
--- a/estado_resultado/TABLERO_Resumen.xlsx
+++ b/estado_resultado/TABLERO_Resumen.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -452,7 +452,7 @@
     <col width="23" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,7 +540,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -549,52 +549,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8950</v>
+        <v>9033</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>21750.07</v>
+        <v>21248.6</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>194663126.5</v>
+        <v>191938603.8</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-7331349</v>
+        <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>199331777.5</v>
+        <v>203938603.8</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.5159861109720238</v>
+        <v>0.5302666766389033</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>186704724.56</v>
+        <v>180204999.95</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>29589894.31563497</v>
+        <v>26342638.17832172</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>-16962841.37563497</v>
+        <v>-2609034.328321721</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>233134.5216142405</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>-17195975.89724921</v>
+        <v>-2609034.328321721</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>-0.08626811095009282</v>
+        <v>-0.01279323423671356</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -603,13 +603,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4681</v>
+        <v>5000</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>23000</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>107663000</v>
+        <v>115000000</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -618,37 +618,37 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>21272182.42</v>
+        <v>14557254</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>128935182.42</v>
+        <v>129557254</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.3337589428979243</v>
+        <v>0.3368655724465751</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>46366452.12</v>
+        <v>62112578.1</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>19139840.46710724</v>
+        <v>16734839.80917067</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>63428889.83289278</v>
+        <v>50709836.09082934</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>150800.0502967046</v>
+        <v>0</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>63278089.78259607</v>
+        <v>50709836.09082934</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>0.4907744232018132</v>
+        <v>0.3914086978937462</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>994</v>
+        <v>1005</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>18331.44</v>
+        <v>17797.52</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>18221451.36</v>
+        <v>17886507.6</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
@@ -672,37 +672,37 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>8719283.16</v>
+        <v>1879283.16</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>26940734.52</v>
+        <v>19765790.76</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.0697382274218899</v>
+        <v>0.0513936056349776</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>14154381.49</v>
+        <v>13033700.32</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>3999229.311203924</v>
+        <v>2553136.407708871</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>8787123.718796074</v>
+        <v>4178954.03229113</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>31509.35256299741</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>8755614.366233077</v>
+        <v>4178954.03229113</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.3249953842102252</v>
+        <v>0.2114235692886152</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -732,31 +732,31 @@
         <v>5339979</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.01382295904566585</v>
+        <v>0.01388463422270195</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>1729983.54</v>
+        <v>940255.37</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>792695.5563204675</v>
+        <v>689762.1737902485</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>2817299.903679532</v>
+        <v>3709961.456209751</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>6245.534280629642</v>
+        <v>0</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>2811054.369398903</v>
+        <v>3709961.456209751</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>0.5264167460956125</v>
+        <v>0.6947520685399233</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -765,13 +765,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>23006</v>
+        <v>23005.72</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>7499865</v>
+        <v>7729921.92</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>0</v>
@@ -783,34 +783,34 @@
         <v>5457100.24</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>12956965.24</v>
+        <v>13187022.16</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.03354013187479501</v>
+        <v>0.03428795865644135</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>8362310.109999999</v>
+        <v>1670327.5</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>3023402.464531557</v>
+        <v>1703360.457204378</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>1571252.665468444</v>
+        <v>9813334.202795623</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>15154.21138909847</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>1556098.454079346</v>
+        <v>9813334.202795623</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.1200974476087539</v>
+        <v>0.7441660508133721</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -840,31 +840,31 @@
         <v>5784313.96</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.01497315532071442</v>
+        <v>0.01503996243503367</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>858655.0569682851</v>
+        <v>747156.6781320452</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>4925658.903031715</v>
+        <v>5037157.281867955</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>6765.219699759979</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>4918893.683331955</v>
+        <v>5037157.281867955</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0.8503849751841539</v>
+        <v>0.8708305456275673</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -894,31 +894,31 @@
         <v>7023340</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.01818047246698663</v>
+        <v>0.01826158996536719</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>1042582.828233555</v>
+        <v>907200.995672081</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>5980757.171766445</v>
+        <v>6116139.004327919</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>8214.360156569415</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>5972542.811609875</v>
+        <v>6116139.004327919</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.8503849751841539</v>
+        <v>0.8708305456275675</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -927,50 +927,50 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14951</v>
+        <v>15374</v>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="n">
-        <v>328047442.86</v>
+        <v>332555033.32</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-7331349</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>53596198.78</v>
+        <v>40041270.36</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>386312292.64</v>
+        <v>384596303.6799999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>257317851.82</v>
+        <v>258013813.48</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>58446300</v>
+        <v>49678094.7</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>70548140.81999996</v>
+        <v>76904395.49999996</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>451823.25</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>70096317.56999996</v>
+        <v>76904395.49999996</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>0.1814498759306164</v>
+        <v>0.1999613484688808</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -979,52 +979,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8893</v>
+        <v>8950</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>21934.95</v>
+        <v>21750.07</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>195067510.35</v>
+        <v>194663126.5</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>-23557895.91</v>
+        <v>-7331349</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>183509614.44</v>
+        <v>199331777.5</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.5079306121308084</v>
+        <v>0.5159861109720238</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>181582548.7</v>
+        <v>216185231.65</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>31220473.13844798</v>
+        <v>29589894.31563497</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>-29293407.39844803</v>
+        <v>-46443348.46563497</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0</v>
+        <v>233134.5216142405</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>-29293407.39844803</v>
+        <v>-46676482.98724921</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>-0.1596287338286886</v>
+        <v>-0.2341647858292399</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1033,13 +1033,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4559</v>
+        <v>4681</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>23000</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>104857000</v>
+        <v>107663000</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>0</v>
@@ -1048,37 +1048,37 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>20638352.53</v>
+        <v>21272182.42</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>125495352.53</v>
+        <v>128935182.42</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.3473547226648214</v>
+        <v>0.3337589428979243</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>82866813.09</v>
+        <v>53726268.12</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>21350512.31304263</v>
+        <v>19139840.46710724</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>21278027.12695737</v>
+        <v>56069073.83289278</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0</v>
+        <v>150800.0502967046</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>21278027.12695737</v>
+        <v>55918273.78259607</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0.169552311683182</v>
+        <v>0.4336929047065296</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1087,10 +1087,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>966</v>
+        <v>994</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>18771.39</v>
+        <v>18331.44</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>18221451.36</v>
@@ -1102,37 +1102,37 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>1879283.16</v>
+        <v>8719283.16</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>20100734.52</v>
+        <v>26940734.52</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.05563620424019061</v>
+        <v>0.0697382274218899</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>6820825.960000001</v>
+        <v>13977106.66</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>3419736.039769831</v>
+        <v>3999229.311203924</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>9860172.520230168</v>
+        <v>8964398.548796074</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0</v>
+        <v>31509.35256299741</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>9860172.520230168</v>
+        <v>8932889.196233077</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.4905379209112687</v>
+        <v>0.3315755622624753</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1156,37 +1156,37 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>6053382.07</v>
+        <v>5339979</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>6053382.07</v>
+        <v>5339979</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.01675496986716224</v>
+        <v>0.01382295904566585</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>2364242.65</v>
+        <v>1729983.54</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>1029861.312116643</v>
+        <v>792695.5563204675</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>2659278.107883357</v>
+        <v>2817299.903679532</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0</v>
+        <v>6245.534280629642</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>2659278.107883357</v>
+        <v>2811054.369398903</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>0.4393045205361302</v>
+        <v>0.5264167460956125</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1195,10 +1195,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>23005.72</v>
+        <v>23006</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>7499865</v>
@@ -1210,37 +1210,37 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>5812890.86</v>
+        <v>5457100.24</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>13312755.86</v>
+        <v>12956965.24</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.03684796708746115</v>
+        <v>0.03354013187479501</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>4725542.23</v>
+        <v>8537787.109999999</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>3364897.880114831</v>
+        <v>3023402.464531557</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>5222315.749885168</v>
+        <v>1395775.665468444</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0</v>
+        <v>15154.21138909847</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>5222315.749885168</v>
+        <v>1380621.454079346</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>0.3922790896794203</v>
+        <v>0.106554384341263</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1264,37 +1264,37 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>5793567.12</v>
+        <v>5784313.96</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>5793567.12</v>
+        <v>5784313.96</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.01603583606593362</v>
+        <v>0.01497315532071442</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>985659.0195436053</v>
+        <v>858655.0569682851</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4807908.100456395</v>
+        <v>4925658.903031715</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0</v>
+        <v>6765.219699759979</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>4807908.100456395</v>
+        <v>4918893.683331955</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>0.8298700957237543</v>
+        <v>0.8503849751841539</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1318,37 +1318,37 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>7023340.5</v>
+        <v>7023340</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>7023340.5</v>
+        <v>7023340</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.01943968794362259</v>
+        <v>0.01818047246698663</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>1194880.246964481</v>
+        <v>1042582.828233555</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>5828460.253035519</v>
+        <v>5980757.171766445</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0</v>
+        <v>8214.360156569415</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>5828460.253035519</v>
+        <v>5972542.811609875</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.8298700957237541</v>
+        <v>0.8503849751841539</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1357,50 +1357,50 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14735</v>
+        <v>14951</v>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="n">
-        <v>325645826.71</v>
+        <v>328047442.86</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>-23557895.91</v>
+        <v>-7331349</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>47200816.24</v>
+        <v>53596198.78</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>361288747.04</v>
+        <v>386312292.64</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>278359972.63</v>
+        <v>294156377.08</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>62566019.95</v>
+        <v>58446300</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>20362754.46000002</v>
+        <v>33709615.56</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0</v>
+        <v>451823.25</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>20362754.46000002</v>
+        <v>33257792.31</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>0.05636144116535566</v>
+        <v>0.08609043238754134</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1409,52 +1409,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>8981</v>
+        <v>8893</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>22121.4</v>
+        <v>21934.95</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>198672293.4</v>
+        <v>195067510.35</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>-17601329.94</v>
+        <v>-23557895.91</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>193070963.46</v>
+        <v>183509614.44</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.5164156772140958</v>
+        <v>0.5079306121308084</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>175827647.74</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>31742016.31813437</v>
+        <v>31220473.13844798</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>161328947.1418656</v>
+        <v>-23538506.43844799</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>161328947.1418656</v>
+        <v>-23538506.43844799</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0.8355940440276997</v>
+        <v>-0.128268518847246</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1484,31 +1484,31 @@
         <v>125495352.53</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.3356681206878028</v>
+        <v>0.3473547226648214</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0</v>
+        <v>138610187</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>20632183.40277549</v>
+        <v>21350512.31304263</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>104863169.1272245</v>
+        <v>-34465346.78304262</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>104863169.1272245</v>
+        <v>-34465346.78304262</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>0.8355940440276997</v>
+        <v>-0.2746344473179084</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1517,13 +1517,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>959</v>
+        <v>966</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>19259.45</v>
+        <v>18771.39</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>18469812.55</v>
+        <v>18221451.36</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -1532,37 +1532,37 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>1973112</v>
+        <v>1879283.16</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>20442924.55</v>
+        <v>20100734.52</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.05467961901952231</v>
+        <v>0.05563620424019061</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>11253777.47</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>3360938.553512358</v>
+        <v>3419736.039769831</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>17081985.99648764</v>
+        <v>5427221.010230169</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>17081985.99648764</v>
+        <v>5427221.010230169</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.8355940440276997</v>
+        <v>0.2700011288060218</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1592,31 +1592,31 @@
         <v>6053382.07</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.01619125602883504</v>
+        <v>0.01675496986716224</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>7280706.05</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>995212.0660839324</v>
+        <v>1029861.312116643</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>5058170.003916068</v>
+        <v>-2257185.292116642</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>5058170.003916068</v>
+        <v>-2257185.292116642</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>0.8355940440276997</v>
+        <v>-0.3728800307026783</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>24823.17</v>
+        <v>23005.72</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>7893768.06</v>
+        <v>7499865</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -1640,37 +1640,37 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>7742890.86</v>
+        <v>5812890.86</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>15636658.92</v>
+        <v>13312755.86</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.04182408198947323</v>
+        <v>0.03684796708746115</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>8720212.65</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>3670759.857955398</v>
+        <v>3364897.880114831</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>11965899.0620446</v>
+        <v>1227645.329885168</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v>11965899.0620446</v>
+        <v>1227645.329885168</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>0.7652465352902</v>
+        <v>0.09221571722604763</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1700,31 +1700,31 @@
         <v>5793567.12</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.01549631717863143</v>
+        <v>0.01603583606593362</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>952496.940853287</v>
+        <v>985659.0195436053</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>4841070.179146713</v>
+        <v>4807908.100456395</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O23" s="2" t="n">
-        <v>4841070.179146713</v>
+        <v>4807908.100456395</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>0.8355940440276995</v>
+        <v>0.8298700957237543</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1748,37 +1748,37 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>7374506.62</v>
+        <v>7023340.5</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>7374506.62</v>
+        <v>7023340.5</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>0.01972492788163938</v>
+        <v>0.01943968794362259</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>1212412.810685158</v>
+        <v>1194880.246964481</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>6162093.809314842</v>
+        <v>5828460.253035519</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>6162093.809314842</v>
+        <v>5828460.253035519</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>0.8355940440276997</v>
+        <v>0.8298700957237541</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1787,50 +1787,50 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>14817</v>
+        <v>14735</v>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="n">
-        <v>329892874.01</v>
+        <v>325645826.71</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>-17601329.94</v>
+        <v>-23557895.91</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>49575811.2</v>
+        <v>47200816.24</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>373867355.27</v>
+        <v>361288747.04</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0</v>
+        <v>355219906.82</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>62566019.95</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>311301335.3200001</v>
+        <v>-56497179.72999997</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>311301335.3200001</v>
+        <v>-56497179.72999997</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>0.8326518240545073</v>
+        <v>-0.1563768044061026</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1839,52 +1839,52 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9030</v>
+        <v>8981</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>22307.22</v>
+        <v>22121.4</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>201434196.6</v>
+        <v>198672293.4</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>-20863268.36</v>
+        <v>-17601329.94</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>192570928.24</v>
+        <v>193070963.46</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.5239744983060236</v>
+        <v>0.5164156772140958</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>222382342.77</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>1336134.97068036</v>
+        <v>31742016.31813437</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>191234793.2693197</v>
+        <v>-61053395.62813437</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O26" s="2" t="n">
-        <v>191234793.2693197</v>
+        <v>-61053395.62813437</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>0.9930615956266506</v>
+        <v>-0.3162225667392149</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1893,13 +1893,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4174</v>
+        <v>4559</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>23000</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>96002000</v>
+        <v>104857000</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -1908,37 +1908,37 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>19577254.16</v>
+        <v>20638352.53</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>115579254.16</v>
+        <v>125495352.53</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.3144845500126275</v>
+        <v>0.3356681206878028</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>110565538.2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>801935.6025322</v>
+        <v>20632183.40277549</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>114777318.5574678</v>
+        <v>-5702369.072775494</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O27" s="2" t="n">
-        <v>114777318.5574678</v>
+        <v>-5702369.072775494</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>0.9930615956266508</v>
+        <v>-0.04543888644332329</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1947,13 +1947,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>927</v>
+        <v>959</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>20087.6</v>
+        <v>19259.45</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>18621205.2</v>
+        <v>18469812.55</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -1962,37 +1962,37 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>5733912</v>
+        <v>1973112</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>24355117.2</v>
+        <v>20442924.55</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.06626888301722196</v>
+        <v>0.05467961901952231</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>10378526.13</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>168985.651693916</v>
+        <v>3360938.553512358</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>24186131.54830608</v>
+        <v>6703459.866487642</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>24186131.54830608</v>
+        <v>6703459.866487642</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>0.9930615956266505</v>
+        <v>0.3279110016813931</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2022,31 +2022,31 @@
         <v>6053382.07</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.01647090691295786</v>
+        <v>0.01619125602883504</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>1045103.78</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>42000.81262804255</v>
+        <v>995212.0660839324</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>6011381.257371957</v>
+        <v>4013066.223916068</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O29" s="2" t="n">
-        <v>6011381.257371957</v>
+        <v>4013066.223916068</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>0.9930615956266506</v>
+        <v>0.6629461311891168</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2055,13 +2055,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>303</v>
+        <v>318</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>24823.17</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>7521420.51</v>
+        <v>7893768.06</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
@@ -2073,34 +2073,34 @@
         <v>7742890.86</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>15264311.37</v>
+        <v>15636658.92</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.0415333195159899</v>
+        <v>0.04182408198947323</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>2703384.4</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>105909.9647657742</v>
+        <v>3670759.857955398</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>15158401.40523423</v>
+        <v>9262514.662044602</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>15158401.40523423</v>
+        <v>9262514.662044602</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>0.9930615956266506</v>
+        <v>0.5923589373812729</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2124,37 +2124,37 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>6322158</v>
+        <v>5793567.12</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>6322158</v>
+        <v>5793567.12</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.01720223086910023</v>
+        <v>0.01549631717863143</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>43865.68871620558</v>
+        <v>952496.940853287</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>6278292.311283794</v>
+        <v>4841070.179146713</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O31" s="2" t="n">
-        <v>6278292.311283794</v>
+        <v>4841070.179146713</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>0.9930615956266506</v>
+        <v>0.8355940440276995</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2184,31 +2184,31 @@
         <v>7374506.62</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.02006561136607911</v>
+        <v>0.01972492788163938</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>51167.30898350174</v>
+        <v>1212412.810685158</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>7323339.311016498</v>
+        <v>6162093.809314842</v>
       </c>
       <c r="N32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>7323339.311016498</v>
+        <v>6162093.809314842</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>0.9930615956266506</v>
+        <v>0.8355940440276997</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mayo 2026</t>
+          <t>Abril 2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2217,44 +2217,474 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>14434</v>
+        <v>14817</v>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="n">
-        <v>323578822.31</v>
+        <v>329892874.01</v>
       </c>
       <c r="F33" s="2" t="n">
         <v>12000000</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>-20863268.36</v>
+        <v>-17601329.94</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>52804103.71</v>
+        <v>49575811.2</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>367519657.66</v>
+        <v>373867355.27</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>347074895.28</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>2550000</v>
+        <v>62566019.95</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>364969657.66</v>
+        <v>-35773559.95999993</v>
       </c>
       <c r="N33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>364969657.66</v>
+        <v>-35773559.95999993</v>
       </c>
       <c r="P33" s="3" t="n">
-        <v>0.9930615956266506</v>
+        <v>-0.0956851660240968</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>OSPEVIC</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>9030</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>22307.22</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>201434196.6</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>-20863268.36</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>192570928.24</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>0.5239744982062241</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>17450261.20128772</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>175120667.0387123</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>175120667.0387123</v>
+      </c>
+      <c r="P34" s="3" t="n">
+        <v>0.9093826811722091</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>OSPIF</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>4174</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>23000</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>96002000</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>19577254.23</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>115579254.23</v>
+      </c>
+      <c r="J35" s="3" t="n">
+        <v>0.3144845501431949</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>10473482.13043821</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>105105772.0995618</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>105105772.0995618</v>
+      </c>
+      <c r="P35" s="3" t="n">
+        <v>0.9093826811722091</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>OSPLYFC</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>927</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>20087.6</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>18621205.2</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>5733912</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>24355117.2</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>0.06626888300459997</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>2206995.420400614</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>22148121.77959938</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>22148121.77959938</v>
+      </c>
+      <c r="P36" s="3" t="n">
+        <v>0.909382681172209</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>OSPM</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>6053382.07</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>6053382.07</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>0.01647090690982071</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>548541.2530236229</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>5504840.816976378</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>5504840.816976378</v>
+      </c>
+      <c r="P37" s="3" t="n">
+        <v>0.9093826811722091</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>OSSURRBAC</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>303</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>24823.17</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>7521420.51</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>7742890.86</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>15264311.37</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>0.0415333195080792</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>1383210.970101964</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>13881100.39989804</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>13881100.39989804</v>
+      </c>
+      <c r="P38" s="3" t="n">
+        <v>0.9093826811722091</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>AMSURRBAC</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>6322158</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>6322158</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>0.01720223086582379</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>572897.0071656689</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>5749260.992834331</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>5749260.992834331</v>
+      </c>
+      <c r="P39" s="3" t="n">
+        <v>0.9093826811722091</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>UOM</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>7374506.62</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>7374506.62</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>0.02006561136225729</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>668258.0175821946</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>6706248.602417805</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>6706248.602417805</v>
+      </c>
+      <c r="P40" s="3" t="n">
+        <v>0.9093826811722091</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Mayo 2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>14434</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="n">
+        <v>323578822.31</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>-20863268.36</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>52804103.78</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>367519657.73</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>33303646</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>334216011.73</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>334216011.73</v>
+      </c>
+      <c r="P41" s="3" t="n">
+        <v>0.9093826811722091</v>
       </c>
     </row>
   </sheetData>
@@ -68256,7 +68686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -68296,11 +68726,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Febrero 2026</t>
+          <t>Enero 2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>451823.25</v>
+        <v>0</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>0</v>
@@ -68309,17 +68739,17 @@
         <v>0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>451823.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Marzo 2026</t>
+          <t>Febrero 2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0</v>
+        <v>451823.25</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>0</v>
@@ -68328,13 +68758,13 @@
         <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>451823.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abril 2026</t>
+          <t>Marzo 2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -68353,19 +68783,38 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Abril 2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Mayo 2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2" t="n">
+      <c r="B6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
actualizar planilla y costos fijos
</commit_message>
<xml_diff>
--- a/estado_resultado/TABLERO_Resumen.xlsx
+++ b/estado_resultado/TABLERO_Resumen.xlsx
@@ -2455,22 +2455,22 @@
         <v>0.01647090690982071</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>6278069.4</v>
+        <v>6115790.4</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>1106330.304429901</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>-1331017.634429901</v>
+        <v>-1168738.634429901</v>
       </c>
       <c r="N37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O37" s="2" t="n">
-        <v>-1331017.634429901</v>
+        <v>-1168738.634429901</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>-0.2198799975019421</v>
+        <v>-0.1930720084929153</v>
       </c>
     </row>
     <row r="38">
@@ -2669,22 +2669,22 @@
         <v>1</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>241954407.27</v>
+        <v>241792128.27</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>67168754.61</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>58396495.85000001</v>
+        <v>58558774.85000001</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O41" s="2" t="n">
-        <v>58396495.85000001</v>
+        <v>58558774.85000001</v>
       </c>
       <c r="P41" s="3" t="n">
-        <v>0.1588935302418606</v>
+        <v>0.1593350821332678</v>
       </c>
     </row>
   </sheetData>
@@ -3422,10 +3422,10 @@
         <v>43</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>102684329.21</v>
+        <v>102522050.21</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>102684329.21</v>
+        <v>102522050.21</v>
       </c>
     </row>
     <row r="35">
@@ -17617,10 +17617,10 @@
         </is>
       </c>
       <c r="C402" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D402" s="2" t="n">
-        <v>21459105.32</v>
+        <v>21219330.52</v>
       </c>
       <c r="E402" s="2" t="n">
         <v>0</v>
@@ -17632,7 +17632,7 @@
         <v>0</v>
       </c>
       <c r="H402" s="2" t="n">
-        <v>21459105.32</v>
+        <v>21219330.52</v>
       </c>
       <c r="I402" t="inlineStr">
         <is>
@@ -17862,10 +17862,10 @@
         </is>
       </c>
       <c r="C409" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D409" s="2" t="n">
-        <v>7130260.82</v>
+        <v>7207756.62</v>
       </c>
       <c r="E409" s="2" t="n">
         <v>0</v>
@@ -17877,7 +17877,7 @@
         <v>0</v>
       </c>
       <c r="H409" s="2" t="n">
-        <v>7130260.82</v>
+        <v>7207756.62</v>
       </c>
       <c r="I409" t="inlineStr">
         <is>
@@ -72412,7 +72412,7 @@
       </c>
       <c r="B1065" t="inlineStr">
         <is>
-          <t>CAMARA DE ENTIDADES DE SALUD - CES</t>
+          <t>SANATORIO DEL SALVADOR PRIVADO SA</t>
         </is>
       </c>
       <c r="C1065" t="inlineStr">
@@ -72444,7 +72444,7 @@
         <v>39</v>
       </c>
       <c r="I1065" s="2" t="n">
-        <v>239774.8</v>
+        <v>77495.8</v>
       </c>
       <c r="J1065" s="2" t="n">
         <v>0</v>
@@ -72453,7 +72453,7 @@
         <v>0</v>
       </c>
       <c r="L1065" s="2" t="n">
-        <v>239774.8</v>
+        <v>77495.8</v>
       </c>
     </row>
     <row r="1066">

</xml_diff>